<commit_message>
Refactor: modularize flashcard app with quiz modes, utils, and UX improvements
- Split monolithic get_words.py into flashcards.py, quiz_modes.py, utils.py
- Add type_answer and article_quiz modes
- Add colorama for colored feedback (green/red/yellow)
- Add input validation, welcome screen, clear screen between questions
- Support umlaut-free input (e.g., 'uber' matches 'über')
- Add requirements.txt

Co-Authored-By: Claude Opus 4
</commit_message>
<xml_diff>
--- a/Vocabular.xlsx
+++ b/Vocabular.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10414"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/awdeshp/Desktop/VER/Code/flashcards_german/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/AWDESHP/Library/CloudStorage/OneDrive-Mercedes-Benz(corpdir.onmicrosoft.com)/Desktop/Academic/flashcards_german/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{650A29EF-A01C-FA40-B1D0-00FC77340E7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D4A023E-792F-F641-A3FB-A7FD2659DD75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13320" yWindow="760" windowWidth="21240" windowHeight="20060" xr2:uid="{8C61D36E-538C-1840-BF80-FF67F9F1A14C}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19760" xr2:uid="{8C61D36E-538C-1840-BF80-FF67F9F1A14C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="447">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="498">
   <si>
     <t>German</t>
   </si>
@@ -1380,6 +1380,160 @@
   </si>
   <si>
     <t xml:space="preserve">It takes considerable efforts to maintain a good relationship. </t>
+  </si>
+  <si>
+    <t>sich dem Ende zuneigen</t>
+  </si>
+  <si>
+    <t>to come to a close</t>
+  </si>
+  <si>
+    <t>The year 2024 is slowly coming to an end.</t>
+  </si>
+  <si>
+    <t>jdn. entlassen</t>
+  </si>
+  <si>
+    <t>to dismiss/fire someone</t>
+  </si>
+  <si>
+    <t>einläuten</t>
+  </si>
+  <si>
+    <t>to herald</t>
+  </si>
+  <si>
+    <t>vorgezogen</t>
+  </si>
+  <si>
+    <t>earlier</t>
+  </si>
+  <si>
+    <t>scheitern (das Scheitern)</t>
+  </si>
+  <si>
+    <t>to fail 
+to fall (government)</t>
+  </si>
+  <si>
+    <t>das Bündnis</t>
+  </si>
+  <si>
+    <t>alliance</t>
+  </si>
+  <si>
+    <t>Das Jahr 2024 neigt sich langsam dem Ende zu.</t>
+  </si>
+  <si>
+    <t>The deeds of his past constantly plagued him.</t>
+  </si>
+  <si>
+    <t>I fell and now have black spots on my arm.</t>
+  </si>
+  <si>
+    <t>One can see many beggars outside Indian temples.</t>
+  </si>
+  <si>
+    <t>The accident was so severe that he injured his vertebral disc.</t>
+  </si>
+  <si>
+    <t>sich erweisen, sich zeigen</t>
+  </si>
+  <si>
+    <t>to turn out</t>
+  </si>
+  <si>
+    <t>Es hat sich herausgestellt, dass die ursprüngliche Diagnose falsch war.</t>
+  </si>
+  <si>
+    <t>It turned out that the original diagnosis was wrong.</t>
+  </si>
+  <si>
+    <t>sich herausstellen</t>
+  </si>
+  <si>
+    <t>ausschlaggebend</t>
+  </si>
+  <si>
+    <t>entscheidend, maßgeblich</t>
+  </si>
+  <si>
+    <t>decisive, determining</t>
+  </si>
+  <si>
+    <t>Der ausschlaggebende Faktor für meine Entscheidung war das Gehalt.</t>
+  </si>
+  <si>
+    <t>The decisive factor for my decision was the salary.</t>
+  </si>
+  <si>
+    <t>nichtsdestotrotz</t>
+  </si>
+  <si>
+    <t>trotzdem, dennoch</t>
+  </si>
+  <si>
+    <t>nevertheless</t>
+  </si>
+  <si>
+    <t>Das Wetter war schlecht; nichtsdestotrotz haben wir die Wanderung gemacht.</t>
+  </si>
+  <si>
+    <t>The weather was bad; nevertheless, we did the hike.</t>
+  </si>
+  <si>
+    <t>scheitern</t>
+  </si>
+  <si>
+    <t>misslingen, fehlschlagen</t>
+  </si>
+  <si>
+    <t>to fail</t>
+  </si>
+  <si>
+    <t>Das Projekt ist an mangelnder Finanzierung gescheitert.</t>
+  </si>
+  <si>
+    <t>The project failed due to lack of funding.</t>
+  </si>
+  <si>
+    <t>behaupten</t>
+  </si>
+  <si>
+    <t>bestreiten, geltend machen</t>
+  </si>
+  <si>
+    <t>to claim, assert</t>
+  </si>
+  <si>
+    <t>Er behauptet, nichts von dem Vorfall gewusst zu haben.</t>
+  </si>
+  <si>
+    <t>He claims to have known nothing about the incident.</t>
+  </si>
+  <si>
+    <t>die Mühe</t>
+  </si>
+  <si>
+    <t>effort, expense</t>
+  </si>
+  <si>
+    <t>Der Aufwand hat sich am Ende gelohnt.</t>
+  </si>
+  <si>
+    <t>The effort paid off in the end.</t>
+  </si>
+  <si>
+    <t>der Aufwand</t>
+  </si>
+  <si>
+    <t>Some actors had to undergo speech therapy in order to speak well.</t>
+  </si>
+  <si>
+    <t>Thanks to the rain, the farmers had a bountiful harvest.</t>
+  </si>
+  <si>
+    <t>He cannot feel his legs after the accident.</t>
   </si>
 </sst>
 </file>
@@ -1438,16 +1592,16 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1763,7 +1917,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A4EFC4A-53BD-EF42-9061-FBB6EFA71DFF}">
-  <dimension ref="A1:E158"/>
+  <dimension ref="A1:E170"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="29.1640625" style="1" customWidth="1"/>
@@ -1809,7 +1963,7 @@
       <c r="C3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="5" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1820,7 +1974,7 @@
       <c r="C4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="6"/>
+      <c r="D4" s="5"/>
     </row>
     <row r="5" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
@@ -1840,8 +1994,11 @@
       <c r="C6" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="5" t="s">
         <v>19</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>464</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1851,7 +2008,7 @@
       <c r="C7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="6"/>
+      <c r="D7" s="5"/>
     </row>
     <row r="8" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
@@ -1874,6 +2031,9 @@
       <c r="D9" s="1" t="s">
         <v>25</v>
       </c>
+      <c r="E9" s="1" t="s">
+        <v>462</v>
+      </c>
     </row>
     <row r="10" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
@@ -1907,10 +2067,10 @@
       <c r="C12" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" s="5" t="s">
         <v>445</v>
       </c>
     </row>
@@ -1921,8 +2081,8 @@
       <c r="C13" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
     </row>
     <row r="14" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
@@ -1953,8 +2113,11 @@
       <c r="C16" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="D16" s="5" t="s">
         <v>47</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>495</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1964,7 +2127,7 @@
       <c r="C17" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D17" s="6"/>
+      <c r="D17" s="5"/>
     </row>
     <row r="18" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
@@ -1973,7 +2136,7 @@
       <c r="C18" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="D18" s="5" t="s">
         <v>52</v>
       </c>
     </row>
@@ -1984,7 +2147,7 @@
       <c r="C19" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D19" s="6"/>
+      <c r="D19" s="5"/>
     </row>
     <row r="20" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
@@ -2018,6 +2181,9 @@
       <c r="D22" s="1" t="s">
         <v>63</v>
       </c>
+      <c r="E22" s="1" t="s">
+        <v>463</v>
+      </c>
     </row>
     <row r="23" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
@@ -2026,8 +2192,11 @@
       <c r="C23" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="D23" s="8" t="s">
+      <c r="D23" s="6" t="s">
         <v>70</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>496</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -2037,7 +2206,8 @@
       <c r="C24" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="D24" s="8"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
     </row>
     <row r="25" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
@@ -2046,7 +2216,8 @@
       <c r="C25" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="D25" s="8"/>
+      <c r="D25" s="6"/>
+      <c r="E25" s="6"/>
     </row>
     <row r="26" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
@@ -2141,7 +2312,7 @@
       <c r="C34" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="D34" s="6" t="s">
+      <c r="D34" s="5" t="s">
         <v>96</v>
       </c>
     </row>
@@ -2152,7 +2323,7 @@
       <c r="C35" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="D35" s="6"/>
+      <c r="D35" s="5"/>
     </row>
     <row r="36" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
@@ -2219,7 +2390,7 @@
       <c r="D41" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="E41" s="6" t="s">
+      <c r="E41" s="5" t="s">
         <v>119</v>
       </c>
     </row>
@@ -2231,7 +2402,7 @@
         <v>115</v>
       </c>
       <c r="D42" s="4"/>
-      <c r="E42" s="6"/>
+      <c r="E42" s="5"/>
     </row>
     <row r="43" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
@@ -2241,7 +2412,7 @@
         <v>117</v>
       </c>
       <c r="D43" s="4"/>
-      <c r="E43" s="6"/>
+      <c r="E43" s="5"/>
     </row>
     <row r="44" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
@@ -2261,7 +2432,7 @@
       <c r="C45" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="D45" s="6" t="s">
+      <c r="D45" s="5" t="s">
         <v>125</v>
       </c>
     </row>
@@ -2272,7 +2443,7 @@
       <c r="C46" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="D46" s="6"/>
+      <c r="D46" s="5"/>
     </row>
     <row r="47" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
@@ -2325,10 +2496,10 @@
       <c r="C51" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="D51" s="6" t="s">
+      <c r="D51" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="E51" s="6" t="s">
+      <c r="E51" s="5" t="s">
         <v>145</v>
       </c>
     </row>
@@ -2339,8 +2510,8 @@
       <c r="C52" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="D52" s="6"/>
-      <c r="E52" s="6"/>
+      <c r="D52" s="5"/>
+      <c r="E52" s="5"/>
     </row>
     <row r="53" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
@@ -2382,7 +2553,7 @@
       <c r="C56" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="D56" s="6" t="s">
+      <c r="D56" s="5" t="s">
         <v>159</v>
       </c>
     </row>
@@ -2393,7 +2564,7 @@
       <c r="C57" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="D57" s="6"/>
+      <c r="D57" s="5"/>
     </row>
     <row r="58" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
@@ -2405,8 +2576,11 @@
       <c r="C58" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="D58" s="6" t="s">
+      <c r="D58" s="5" t="s">
         <v>165</v>
+      </c>
+      <c r="E58" s="5" t="s">
+        <v>497</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -2416,7 +2590,8 @@
       <c r="C59" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="D59" s="6"/>
+      <c r="D59" s="5"/>
+      <c r="E59" s="5"/>
     </row>
     <row r="60" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
@@ -2567,7 +2742,7 @@
       <c r="C73" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="D73" s="6" t="s">
+      <c r="D73" s="5" t="s">
         <v>201</v>
       </c>
     </row>
@@ -2578,7 +2753,7 @@
       <c r="C74" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="D74" s="6"/>
+      <c r="D74" s="5"/>
     </row>
     <row r="75" spans="1:5" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
@@ -2587,7 +2762,7 @@
       <c r="C75" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="D75" s="6" t="s">
+      <c r="D75" s="5" t="s">
         <v>208</v>
       </c>
     </row>
@@ -2598,7 +2773,7 @@
       <c r="C76" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="D76" s="6"/>
+      <c r="D76" s="5"/>
     </row>
     <row r="77" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
@@ -2607,7 +2782,7 @@
       <c r="C77" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="D77" s="7" t="s">
+      <c r="D77" s="8" t="s">
         <v>213</v>
       </c>
     </row>
@@ -2618,7 +2793,7 @@
       <c r="C78" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="D78" s="7"/>
+      <c r="D78" s="8"/>
     </row>
     <row r="79" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="s">
@@ -2638,10 +2813,10 @@
       <c r="C80" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="D80" s="6" t="s">
+      <c r="D80" s="5" t="s">
         <v>221</v>
       </c>
-      <c r="E80" s="6" t="s">
+      <c r="E80" s="5" t="s">
         <v>444</v>
       </c>
     </row>
@@ -2652,8 +2827,8 @@
       <c r="C81" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="D81" s="6"/>
-      <c r="E81" s="6"/>
+      <c r="D81" s="5"/>
+      <c r="E81" s="5"/>
     </row>
     <row r="82" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A82" s="1" t="s">
@@ -2695,7 +2870,7 @@
       <c r="C85" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="D85" s="6" t="s">
+      <c r="D85" s="5" t="s">
         <v>235</v>
       </c>
     </row>
@@ -2706,7 +2881,7 @@
       <c r="C86" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="D86" s="6"/>
+      <c r="D86" s="5"/>
     </row>
     <row r="87" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A87" s="1" t="s">
@@ -2715,7 +2890,7 @@
       <c r="C87" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="D87" s="6" t="s">
+      <c r="D87" s="5" t="s">
         <v>240</v>
       </c>
     </row>
@@ -2726,7 +2901,7 @@
       <c r="C88" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="D88" s="6"/>
+      <c r="D88" s="5"/>
     </row>
     <row r="89" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A89" s="1" t="s">
@@ -2768,7 +2943,7 @@
       <c r="C92" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="D92" s="6" t="s">
+      <c r="D92" s="5" t="s">
         <v>254</v>
       </c>
     </row>
@@ -2779,7 +2954,7 @@
       <c r="C93" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="D93" s="6"/>
+      <c r="D93" s="5"/>
     </row>
     <row r="94" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A94" s="1" t="s">
@@ -2799,7 +2974,7 @@
       <c r="C95" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="D95" s="6" t="s">
+      <c r="D95" s="5" t="s">
         <v>262</v>
       </c>
     </row>
@@ -2810,7 +2985,7 @@
       <c r="C96" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="D96" s="6"/>
+      <c r="D96" s="5"/>
     </row>
     <row r="97" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A97" s="1" t="s">
@@ -2819,7 +2994,7 @@
       <c r="C97" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="D97" s="6" t="s">
+      <c r="D97" s="5" t="s">
         <v>267</v>
       </c>
     </row>
@@ -2830,7 +3005,7 @@
       <c r="C98" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="D98" s="6"/>
+      <c r="D98" s="5"/>
     </row>
     <row r="99" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A99" s="1" t="s">
@@ -2955,6 +3130,9 @@
       <c r="D109" s="1" t="s">
         <v>297</v>
       </c>
+      <c r="E109" s="1" t="s">
+        <v>461</v>
+      </c>
     </row>
     <row r="110" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A110" s="1" t="s">
@@ -2996,7 +3174,7 @@
       <c r="C113" s="1" t="s">
         <v>308</v>
       </c>
-      <c r="D113" s="6" t="s">
+      <c r="D113" s="5" t="s">
         <v>310</v>
       </c>
     </row>
@@ -3007,7 +3185,7 @@
       <c r="C114" s="1" t="s">
         <v>309</v>
       </c>
-      <c r="D114" s="6"/>
+      <c r="D114" s="5"/>
     </row>
     <row r="115" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A115" s="1" t="s">
@@ -3016,7 +3194,7 @@
       <c r="C115" s="1" t="s">
         <v>312</v>
       </c>
-      <c r="D115" s="6" t="s">
+      <c r="D115" s="5" t="s">
         <v>315</v>
       </c>
     </row>
@@ -3027,7 +3205,7 @@
       <c r="C116" s="1" t="s">
         <v>314</v>
       </c>
-      <c r="D116" s="6"/>
+      <c r="D116" s="5"/>
     </row>
     <row r="117" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A117" s="1" t="s">
@@ -3167,7 +3345,7 @@
       <c r="C129" s="1" t="s">
         <v>352</v>
       </c>
-      <c r="D129" s="5" t="s">
+      <c r="D129" s="7" t="s">
         <v>355</v>
       </c>
     </row>
@@ -3178,7 +3356,7 @@
       <c r="C130" s="1" t="s">
         <v>354</v>
       </c>
-      <c r="D130" s="5"/>
+      <c r="D130" s="7"/>
     </row>
     <row r="131" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A131" s="1" t="s">
@@ -3507,8 +3685,197 @@
       <c r="D158" s="4"/>
       <c r="E158" s="4"/>
     </row>
+    <row r="159" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A159" s="1" t="s">
+        <v>447</v>
+      </c>
+      <c r="C159" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="D159" s="1" t="s">
+        <v>460</v>
+      </c>
+      <c r="E159" s="1" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="160" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A160" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="C160" s="1" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="161" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A161" s="1" t="s">
+        <v>452</v>
+      </c>
+      <c r="C161" s="1" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="162" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A162" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="C162" s="1" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="163" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A163" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="C163" s="1" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A164" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="C164" s="1" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="165" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A165" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B165" s="1" t="s">
+        <v>465</v>
+      </c>
+      <c r="C165" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="D165" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="E165" s="1" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="166" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A166" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="B166" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="C166" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="D166" s="1" t="s">
+        <v>473</v>
+      </c>
+      <c r="E166" s="1" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="167" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A167" s="1" t="s">
+        <v>475</v>
+      </c>
+      <c r="B167" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="C167" s="1" t="s">
+        <v>477</v>
+      </c>
+      <c r="D167" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="E167" s="1" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="168" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A168" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="B168" s="1" t="s">
+        <v>481</v>
+      </c>
+      <c r="C168" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="D168" s="1" t="s">
+        <v>483</v>
+      </c>
+      <c r="E168" s="1" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="169" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A169" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="B169" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="C169" s="1" t="s">
+        <v>487</v>
+      </c>
+      <c r="D169" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="E169" s="1" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A170" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="B170" s="1" t="s">
+        <v>490</v>
+      </c>
+      <c r="C170" s="1" t="s">
+        <v>491</v>
+      </c>
+      <c r="D170" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="E170" s="1" t="s">
+        <v>493</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="47">
+  <mergeCells count="49">
+    <mergeCell ref="E23:E25"/>
+    <mergeCell ref="E58:E59"/>
+    <mergeCell ref="D145:D146"/>
+    <mergeCell ref="E145:E146"/>
+    <mergeCell ref="D137:D138"/>
+    <mergeCell ref="D139:D140"/>
+    <mergeCell ref="D141:D142"/>
+    <mergeCell ref="D26:D27"/>
+    <mergeCell ref="E104:E107"/>
+    <mergeCell ref="E120:E122"/>
+    <mergeCell ref="E141:E142"/>
+    <mergeCell ref="D120:D122"/>
+    <mergeCell ref="D67:D71"/>
+    <mergeCell ref="D127:D128"/>
+    <mergeCell ref="D129:D130"/>
+    <mergeCell ref="D131:D133"/>
+    <mergeCell ref="E41:E43"/>
+    <mergeCell ref="D73:D74"/>
+    <mergeCell ref="D75:D76"/>
+    <mergeCell ref="D77:D78"/>
+    <mergeCell ref="D80:D81"/>
+    <mergeCell ref="D45:D46"/>
+    <mergeCell ref="D51:D52"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="D95:D96"/>
+    <mergeCell ref="D97:D98"/>
+    <mergeCell ref="E51:E52"/>
+    <mergeCell ref="D56:D57"/>
+    <mergeCell ref="D58:D59"/>
     <mergeCell ref="D155:D158"/>
     <mergeCell ref="E155:E158"/>
     <mergeCell ref="E80:E81"/>
@@ -3525,37 +3892,6 @@
     <mergeCell ref="D85:D86"/>
     <mergeCell ref="D87:D88"/>
     <mergeCell ref="D92:D93"/>
-    <mergeCell ref="D95:D96"/>
-    <mergeCell ref="D97:D98"/>
-    <mergeCell ref="E51:E52"/>
-    <mergeCell ref="D56:D57"/>
-    <mergeCell ref="D58:D59"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="D26:D27"/>
-    <mergeCell ref="E104:E107"/>
-    <mergeCell ref="E120:E122"/>
-    <mergeCell ref="E141:E142"/>
-    <mergeCell ref="D120:D122"/>
-    <mergeCell ref="D67:D71"/>
-    <mergeCell ref="D127:D128"/>
-    <mergeCell ref="D129:D130"/>
-    <mergeCell ref="D131:D133"/>
-    <mergeCell ref="E41:E43"/>
-    <mergeCell ref="D73:D74"/>
-    <mergeCell ref="D75:D76"/>
-    <mergeCell ref="D77:D78"/>
-    <mergeCell ref="D80:D81"/>
-    <mergeCell ref="D45:D46"/>
-    <mergeCell ref="D51:D52"/>
-    <mergeCell ref="D145:D146"/>
-    <mergeCell ref="E145:E146"/>
-    <mergeCell ref="D137:D138"/>
-    <mergeCell ref="D139:D140"/>
-    <mergeCell ref="D141:D142"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>